<commit_message>
feat (sercured_webshop) : Implémenter l’utilisation d’un token JWT
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_Chabal.xlsx
+++ b/Journal-de-Travail_Chabal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3019223A-ABA0-43CC-BB13-C47F06442BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E19818-E548-41BF-BC05-C65A5F038037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="6570" yWindow="345" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
   <si>
     <t>Auteur:</t>
   </si>
@@ -147,6 +147,9 @@
   <si>
     <t>Ajoute du hash des mdp, du sel, du poivre</t>
   </si>
+  <si>
+    <t>Implémenter l’utilisation d’un token JWT</t>
+  </si>
 </sst>
 </file>
 
@@ -159,7 +162,7 @@
     <numFmt numFmtId="167" formatCode="dd\ mmm"/>
     <numFmt numFmtId="168" formatCode="00\ &quot;min&quot;"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -275,6 +278,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -380,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -575,6 +584,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1088,7 +1101,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>270</c:v>
+                  <c:v>315</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4181,7 +4194,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>4 heures 30 minutes</v>
+        <v>5 heures 15 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4200,11 +4213,11 @@
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>150</v>
+        <v>195</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4349,16 +4362,24 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="74" t="str">
+    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="74">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="40"/>
+        <v>17</v>
+      </c>
+      <c r="B11" s="40">
+        <v>46136</v>
+      </c>
       <c r="C11" s="41"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="28"/>
+      <c r="D11" s="42">
+        <v>45</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="83" t="s">
+        <v>35</v>
+      </c>
       <c r="G11" s="46"/>
       <c r="M11" t="s">
         <v>4</v>
@@ -10830,11 +10851,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>150</v>
+        <v>195</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10842,7 +10863,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>4 h 30 min</v>
+        <v>5 h 15 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -10941,22 +10962,22 @@
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>150</v>
+        <v>195</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>4 h 30 min</v>
+        <v>5 h 15 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>5.113636363636364E-2</v>
+        <v>5.9659090909090912E-2</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -10995,18 +11016,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11219,6 +11228,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11229,19 +11250,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11260,6 +11268,19 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat (sercured_webshop) : Ajouter les rôles administrateur et utilisateur dans le JWT et protéger les routes d’administration
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_Chabal.xlsx
+++ b/Journal-de-Travail_Chabal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E19818-E548-41BF-BC05-C65A5F038037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441AA691-7CE2-4BD6-BC61-FA0950D9DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6570" yWindow="345" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
   <si>
     <t>Auteur:</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>Implémenter l’utilisation d’un token JWT</t>
+  </si>
+  <si>
+    <t>Ajouter les rôles administrateur et utilisateur dans le JWT et protéger les routes d’administration</t>
   </si>
 </sst>
 </file>
@@ -575,6 +578,10 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="16" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -584,10 +591,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1101,7 +1104,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>315</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4171,15 +4174,15 @@
       <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="80" t="s">
+      <c r="B2" s="83"/>
+      <c r="C2" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
       <c r="F2" s="5" t="s">
         <v>1</v>
       </c>
@@ -4188,13 +4191,13 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="82"/>
+      <c r="B3" s="83"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>5 heures 15 minutes</v>
+        <v>6 heures 0 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4213,20 +4216,20 @@
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C5" s="81" t="s">
+      <c r="C5" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="81"/>
+      <c r="D5" s="82"/>
     </row>
     <row r="6" spans="1:15" s="17" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
@@ -4377,7 +4380,7 @@
       <c r="E11" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="83" t="s">
+      <c r="F11" s="80" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="46"/>
@@ -4392,15 +4395,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="73" t="str">
+      <c r="A12" s="73">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="36"/>
+        <v>17</v>
+      </c>
+      <c r="B12" s="36">
+        <v>46136</v>
+      </c>
       <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="28"/>
+      <c r="D12" s="38">
+        <v>45</v>
+      </c>
+      <c r="E12" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>36</v>
+      </c>
       <c r="G12" s="45"/>
       <c r="N12">
         <v>5</v>
@@ -10851,11 +10862,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10863,7 +10874,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>5 h 15 min</v>
+        <v>6 h 00 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -10962,22 +10973,22 @@
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 15 min</v>
+        <v>6 h 00 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>5.9659090909090912E-2</v>
+        <v>6.8181818181818177E-2</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11016,6 +11027,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11228,18 +11251,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11250,6 +11261,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11268,19 +11292,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>